<commit_message>
feat: added module list readme feat: updated module list excel feat: added export_modules.py for converting excel to CSV
</commit_message>
<xml_diff>
--- a/docs/module_list.xlsx
+++ b/docs/module_list.xlsx
@@ -126,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -240,6 +240,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -605,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J38"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -615,8 +624,8 @@
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="42" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
     <col width="38" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -658,15 +667,25 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>RotationMode</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Clearance</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -706,17 +725,25 @@
       <c r="G2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>AlignToRoad</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Marketplace</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>2-3 storey, primary residential filler</t>
         </is>
@@ -756,17 +783,25 @@
       <c r="G3" s="3" t="n">
         <v>0.6</v>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>AlignToRoad</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Marketplace</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>4-6 storey, skyline variation</t>
         </is>
@@ -806,17 +841,25 @@
       <c r="G4" s="3" t="n">
         <v>0.4</v>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>AlignToRoad</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
         <is>
           <t>Marketplace</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="L4" s="4" t="inlineStr">
         <is>
           <t>Stepped housing, hero belt</t>
         </is>
@@ -856,17 +899,25 @@
       <c r="G5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>AlignToRoad</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>Marketplace</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>Large footprint, low detail</t>
         </is>
@@ -906,17 +957,25 @@
       <c r="G6" s="3" t="n">
         <v>0.5</v>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>AlignToRoad</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>Marketplace</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="L6" s="4" t="inlineStr">
         <is>
           <t>Tanks/stacks, reads at distance</t>
         </is>
@@ -956,17 +1015,25 @@
       <c r="G7" s="3" t="n">
         <v>0.8</v>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>AlignToRoad</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Marketplace</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>Street-level commercial</t>
         </is>
@@ -1006,17 +1073,25 @@
       <c r="G8" s="3" t="n">
         <v>0.6</v>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>AlignToRoad</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>Marketplace</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="L8" s="4" t="inlineStr">
         <is>
           <t>Small civic structure</t>
         </is>
@@ -1056,17 +1131,25 @@
       <c r="G9" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="K9" s="5" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J9" s="7" t="inlineStr">
+      <c r="L9" s="7" t="inlineStr">
         <is>
           <t>Primary repeating rib along belt</t>
         </is>
@@ -1106,17 +1189,25 @@
       <c r="G10" s="6" t="n">
         <v>0.4</v>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="K10" s="5" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J10" s="7" t="inlineStr">
+      <c r="L10" s="7" t="inlineStr">
         <is>
           <t>Where ribs meet belt boundaries</t>
         </is>
@@ -1156,17 +1247,25 @@
       <c r="G11" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="K11" s="5" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J11" s="7" t="inlineStr">
+      <c r="L11" s="7" t="inlineStr">
         <is>
           <t>Main tiling floor plate</t>
         </is>
@@ -1206,17 +1305,25 @@
       <c r="G12" s="6" t="n">
         <v>0.5</v>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="K12" s="5" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J12" s="7" t="inlineStr">
+      <c r="L12" s="7" t="inlineStr">
         <is>
           <t>Direction changes</t>
         </is>
@@ -1256,17 +1363,25 @@
       <c r="G13" s="6" t="n">
         <v>0.7</v>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="K13" s="5" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J13" s="7" t="inlineStr">
+      <c r="L13" s="7" t="inlineStr">
         <is>
           <t>Vertical structural member</t>
         </is>
@@ -1306,17 +1421,25 @@
       <c r="G14" s="6" t="n">
         <v>0.5</v>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="K14" s="5" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J14" s="7" t="inlineStr">
+      <c r="L14" s="7" t="inlineStr">
         <is>
           <t>Breaks long runs, belt divider</t>
         </is>
@@ -1356,17 +1479,25 @@
       <c r="G15" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H15" s="8" t="inlineStr">
+      <c r="H15" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="8" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="I15" s="8" t="inlineStr">
+      <c r="K15" s="8" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J15" s="10" t="inlineStr">
+      <c r="L15" s="10" t="inlineStr">
         <is>
           <t>Primary walkable surface</t>
         </is>
@@ -1406,17 +1537,25 @@
       <c r="G16" s="9" t="n">
         <v>0.5</v>
       </c>
-      <c r="H16" s="8" t="inlineStr">
+      <c r="H16" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I16" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="8" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="I16" s="8" t="inlineStr">
+      <c r="K16" s="8" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J16" s="10" t="inlineStr">
+      <c r="L16" s="10" t="inlineStr">
         <is>
           <t>Hero belt open space</t>
         </is>
@@ -1456,17 +1595,25 @@
       <c r="G17" s="9" t="n">
         <v>0.8</v>
       </c>
-      <c r="H17" s="8" t="inlineStr">
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="8" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="I17" s="8" t="inlineStr">
+      <c r="K17" s="8" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J17" s="10" t="inlineStr">
+      <c r="L17" s="10" t="inlineStr">
         <is>
           <t>Green ground variant</t>
         </is>
@@ -1506,17 +1653,25 @@
       <c r="G18" s="9" t="n">
         <v>0.6</v>
       </c>
-      <c r="H18" s="8" t="inlineStr">
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I18" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="8" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="I18" s="8" t="inlineStr">
+      <c r="K18" s="8" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J18" s="10" t="inlineStr">
+      <c r="L18" s="10" t="inlineStr">
         <is>
           <t>Blend paved to planted</t>
         </is>
@@ -1556,17 +1711,25 @@
       <c r="G19" s="9" t="n">
         <v>0.9</v>
       </c>
-      <c r="H19" s="8" t="inlineStr">
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="I19" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="8" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="I19" s="8" t="inlineStr">
+      <c r="K19" s="8" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J19" s="10" t="inlineStr">
+      <c r="L19" s="10" t="inlineStr">
         <is>
           <t>Connective walkway</t>
         </is>
@@ -1606,17 +1769,25 @@
       <c r="G20" s="12" t="n">
         <v>0.4</v>
       </c>
-      <c r="H20" s="11" t="inlineStr">
+      <c r="H20" s="12" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I20" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="11" t="inlineStr">
         <is>
           <t>Megascans</t>
         </is>
       </c>
-      <c r="I20" s="11" t="inlineStr">
+      <c r="K20" s="11" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J20" s="13" t="inlineStr">
+      <c r="L20" s="13" t="inlineStr">
         <is>
           <t>Hero belt focal planting</t>
         </is>
@@ -1656,17 +1827,25 @@
       <c r="G21" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H21" s="11" t="inlineStr">
+      <c r="H21" s="12" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I21" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" s="11" t="inlineStr">
         <is>
           <t>Megascans</t>
         </is>
       </c>
-      <c r="I21" s="11" t="inlineStr">
+      <c r="K21" s="11" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J21" s="13" t="inlineStr">
+      <c r="L21" s="13" t="inlineStr">
         <is>
           <t>Primary scatter tree</t>
         </is>
@@ -1706,17 +1885,25 @@
       <c r="G22" s="12" t="n">
         <v>0.6</v>
       </c>
-      <c r="H22" s="11" t="inlineStr">
+      <c r="H22" s="12" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I22" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="11" t="inlineStr">
         <is>
           <t>Megascans</t>
         </is>
       </c>
-      <c r="I22" s="11" t="inlineStr">
+      <c r="K22" s="11" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J22" s="13" t="inlineStr">
+      <c r="L22" s="13" t="inlineStr">
         <is>
           <t>Silhouette variation</t>
         </is>
@@ -1756,17 +1943,25 @@
       <c r="G23" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H23" s="11" t="inlineStr">
+      <c r="H23" s="12" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I23" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J23" s="11" t="inlineStr">
         <is>
           <t>Megascans</t>
         </is>
       </c>
-      <c r="I23" s="11" t="inlineStr">
+      <c r="K23" s="11" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J23" s="13" t="inlineStr">
+      <c r="L23" s="13" t="inlineStr">
         <is>
           <t>Mid-layer scatter</t>
         </is>
@@ -1806,17 +2001,25 @@
       <c r="G24" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H24" s="11" t="inlineStr">
+      <c r="H24" s="12" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I24" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" s="11" t="inlineStr">
         <is>
           <t>Megascans</t>
         </is>
       </c>
-      <c r="I24" s="11" t="inlineStr">
+      <c r="K24" s="11" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J24" s="13" t="inlineStr">
+      <c r="L24" s="13" t="inlineStr">
         <is>
           <t>Dense scatter filler</t>
         </is>
@@ -1856,17 +2059,25 @@
       <c r="G25" s="12" t="n">
         <v>0.7</v>
       </c>
-      <c r="H25" s="11" t="inlineStr">
+      <c r="H25" s="12" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I25" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J25" s="11" t="inlineStr">
         <is>
           <t>Megascans</t>
         </is>
       </c>
-      <c r="I25" s="11" t="inlineStr">
+      <c r="K25" s="11" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J25" s="13" t="inlineStr">
+      <c r="L25" s="13" t="inlineStr">
         <is>
           <t>Undergrowth variation</t>
         </is>
@@ -1906,17 +2117,25 @@
       <c r="G26" s="12" t="n">
         <v>0.8</v>
       </c>
-      <c r="H26" s="11" t="inlineStr">
+      <c r="H26" s="12" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I26" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J26" s="11" t="inlineStr">
         <is>
           <t>Megascans</t>
         </is>
       </c>
-      <c r="I26" s="11" t="inlineStr">
+      <c r="K26" s="11" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J26" s="13" t="inlineStr">
+      <c r="L26" s="13" t="inlineStr">
         <is>
           <t>Agriculture belt</t>
         </is>
@@ -1956,17 +2175,25 @@
       <c r="G27" s="12" t="n">
         <v>0.5</v>
       </c>
-      <c r="H27" s="11" t="inlineStr">
+      <c r="H27" s="12" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I27" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J27" s="11" t="inlineStr">
         <is>
           <t>Marketplace</t>
         </is>
       </c>
-      <c r="I27" s="11" t="inlineStr">
+      <c r="K27" s="11" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J27" s="13" t="inlineStr">
+      <c r="L27" s="13" t="inlineStr">
         <is>
           <t>Urban greenery, hero belt</t>
         </is>
@@ -2006,17 +2233,25 @@
       <c r="G28" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="H28" s="14" t="inlineStr">
+      <c r="H28" s="15" t="inlineStr">
+        <is>
+          <t>AlignToRoad</t>
+        </is>
+      </c>
+      <c r="I28" s="15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J28" s="14" t="inlineStr">
         <is>
           <t>Marketplace</t>
         </is>
       </c>
-      <c r="I28" s="14" t="inlineStr">
+      <c r="K28" s="14" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J28" s="16" t="inlineStr">
+      <c r="L28" s="16" t="inlineStr">
         <is>
           <t>Primary run</t>
         </is>
@@ -2056,17 +2291,25 @@
       <c r="G29" s="15" t="n">
         <v>0.6</v>
       </c>
-      <c r="H29" s="14" t="inlineStr">
+      <c r="H29" s="15" t="inlineStr">
+        <is>
+          <t>AlignToRoad</t>
+        </is>
+      </c>
+      <c r="I29" s="15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J29" s="14" t="inlineStr">
         <is>
           <t>Marketplace</t>
         </is>
       </c>
-      <c r="I29" s="14" t="inlineStr">
+      <c r="K29" s="14" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J29" s="16" t="inlineStr">
+      <c r="L29" s="16" t="inlineStr">
         <is>
           <t>Direction change</t>
         </is>
@@ -2106,17 +2349,25 @@
       <c r="G30" s="15" t="n">
         <v>0.8</v>
       </c>
-      <c r="H30" s="14" t="inlineStr">
+      <c r="H30" s="15" t="inlineStr">
+        <is>
+          <t>AlignToRoad</t>
+        </is>
+      </c>
+      <c r="I30" s="15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J30" s="14" t="inlineStr">
         <is>
           <t>Marketplace</t>
         </is>
       </c>
-      <c r="I30" s="14" t="inlineStr">
+      <c r="K30" s="14" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J30" s="16" t="inlineStr">
+      <c r="L30" s="16" t="inlineStr">
         <is>
           <t>Surface detail, high reuse</t>
         </is>
@@ -2156,17 +2407,25 @@
       <c r="G31" s="15" t="n">
         <v>0.9</v>
       </c>
-      <c r="H31" s="14" t="inlineStr">
+      <c r="H31" s="15" t="inlineStr">
+        <is>
+          <t>AlignToRoad</t>
+        </is>
+      </c>
+      <c r="I31" s="15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J31" s="14" t="inlineStr">
         <is>
           <t>Marketplace</t>
         </is>
       </c>
-      <c r="I31" s="14" t="inlineStr">
+      <c r="K31" s="14" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J31" s="16" t="inlineStr">
+      <c r="L31" s="16" t="inlineStr">
         <is>
           <t>Emissive, drives night read</t>
         </is>
@@ -2206,17 +2465,25 @@
       <c r="G32" s="15" t="n">
         <v>0.7</v>
       </c>
-      <c r="H32" s="14" t="inlineStr">
+      <c r="H32" s="15" t="inlineStr">
+        <is>
+          <t>AlignToRoad</t>
+        </is>
+      </c>
+      <c r="I32" s="15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J32" s="14" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="I32" s="14" t="inlineStr">
+      <c r="K32" s="14" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J32" s="16" t="inlineStr">
+      <c r="L32" s="16" t="inlineStr">
         <is>
           <t>Emissive, simple geometry</t>
         </is>
@@ -2256,17 +2523,25 @@
       <c r="G33" s="15" t="n">
         <v>0.8</v>
       </c>
-      <c r="H33" s="14" t="inlineStr">
+      <c r="H33" s="15" t="inlineStr">
+        <is>
+          <t>AlignToRoad</t>
+        </is>
+      </c>
+      <c r="I33" s="15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J33" s="14" t="inlineStr">
         <is>
           <t>Marketplace</t>
         </is>
       </c>
-      <c r="I33" s="14" t="inlineStr">
+      <c r="K33" s="14" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J33" s="16" t="inlineStr">
+      <c r="L33" s="16" t="inlineStr">
         <is>
           <t>Connective tissue</t>
         </is>
@@ -2306,17 +2581,25 @@
       <c r="G34" s="15" t="n">
         <v>0.7</v>
       </c>
-      <c r="H34" s="14" t="inlineStr">
+      <c r="H34" s="15" t="inlineStr">
+        <is>
+          <t>AlignToRoad</t>
+        </is>
+      </c>
+      <c r="I34" s="15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J34" s="14" t="inlineStr">
         <is>
           <t>Marketplace</t>
         </is>
       </c>
-      <c r="I34" s="14" t="inlineStr">
+      <c r="K34" s="14" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J34" s="16" t="inlineStr">
+      <c r="L34" s="16" t="inlineStr">
         <is>
           <t>Small scatter detail</t>
         </is>
@@ -2356,17 +2639,25 @@
       <c r="G35" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="H35" s="17" t="inlineStr">
+      <c r="H35" s="18" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I35" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" s="17" t="inlineStr">
         <is>
           <t>Scan</t>
         </is>
       </c>
-      <c r="I35" s="17" t="inlineStr">
+      <c r="K35" s="17" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J35" s="19" t="inlineStr">
+      <c r="L35" s="19" t="inlineStr">
         <is>
           <t>SELF-SCANNED - photogrammetry piece</t>
         </is>
@@ -2406,17 +2697,25 @@
       <c r="G36" s="18" t="n">
         <v>0.8</v>
       </c>
-      <c r="H36" s="17" t="inlineStr">
+      <c r="H36" s="18" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I36" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" s="17" t="inlineStr">
         <is>
           <t>Marketplace</t>
         </is>
       </c>
-      <c r="I36" s="17" t="inlineStr">
+      <c r="K36" s="17" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J36" s="19" t="inlineStr">
+      <c r="L36" s="19" t="inlineStr">
         <is>
           <t>Edge/corner accumulation</t>
         </is>
@@ -2456,17 +2755,25 @@
       <c r="G37" s="18" t="n">
         <v>0.7</v>
       </c>
-      <c r="H37" s="17" t="inlineStr">
+      <c r="H37" s="18" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I37" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" s="17" t="inlineStr">
         <is>
           <t>Marketplace</t>
         </is>
       </c>
-      <c r="I37" s="17" t="inlineStr">
+      <c r="K37" s="17" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J37" s="19" t="inlineStr">
+      <c r="L37" s="19" t="inlineStr">
         <is>
           <t>Reads as inhabited</t>
         </is>
@@ -2506,24 +2813,32 @@
       <c r="G38" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="H38" s="17" t="inlineStr">
+      <c r="H38" s="18" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="I38" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="17" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="I38" s="17" t="inlineStr">
+      <c r="K38" s="17" t="inlineStr">
         <is>
           <t>Not Started</t>
         </is>
       </c>
-      <c r="J38" s="19" t="inlineStr">
+      <c r="L38" s="19" t="inlineStr">
         <is>
           <t>Blended into M_Structural grime</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
+  <dataValidations count="7">
     <dataValidation sqref="D2:D38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Residential,Industrial,Service,-"</formula1>
     </dataValidation>
@@ -2540,6 +2855,12 @@
       <formula1>0</formula1>
       <formula2>1</formula2>
     </dataValidation>
+    <dataValidation sqref="H2:H38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Free,AlignToRoad,Fixed"</formula1>
+    </dataValidation>
+    <dataValidation sqref="I2:I38" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="decimal" operator="greaterThanOrEqual">
+      <formula1>0</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2551,7 +2872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2954,6 +3275,70 @@
       <c r="B16" s="40" t="inlineStr">
         <is>
           <t>For humans only. Change it freely, nothing breaks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="58" customHeight="1">
+      <c r="A17" s="43" t="inlineStr">
+        <is>
+          <t>RotationMode</t>
+        </is>
+      </c>
+      <c r="B17" s="28" t="inlineStr">
+        <is>
+          <t>Whether this module can be rotated freely when placed, or must face something. PCG cannot infer intent - a tree can face anywhere, a shopfront cannot.</t>
+        </is>
+      </c>
+      <c r="C17" s="44" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+      <c r="D17" s="44" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="E17" s="28" t="inlineStr">
+        <is>
+          <t>Free = any yaw. AlignToRoad = must face the nearest street. Fixed = placed at authored rotation only. NOTE: these values are a first draft - the PCG graph may want different categories once built.</t>
+        </is>
+      </c>
+      <c r="F17" s="45" t="inlineStr">
+        <is>
+          <t>AlignToRoad</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="58" customHeight="1">
+      <c r="A18" s="43" t="inlineStr">
+        <is>
+          <t>Clearance</t>
+        </is>
+      </c>
+      <c r="B18" s="28" t="inlineStr">
+        <is>
+          <t>Extra space in metres this module needs beyond its own mesh bounds. PCG's Bounds Modifier already prevents literal overlap; this is for breathing room.</t>
+        </is>
+      </c>
+      <c r="C18" s="44" t="inlineStr">
+        <is>
+          <t>Artist</t>
+        </is>
+      </c>
+      <c r="D18" s="44" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="E18" s="28" t="inlineStr">
+        <is>
+          <t>Metres, 0 or greater. 0 means the mesh bounds are enough. A warehouse might want 5. Too high and the belt looks sparse; too low and it looks cluttered.</t>
+        </is>
+      </c>
+      <c r="F18" s="45" t="inlineStr">
+        <is>
+          <t>2.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: added DT modules and added s modules feat: added PCG for testing
</commit_message>
<xml_diff>
--- a/docs/module_list.xlsx
+++ b/docs/module_list.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Module List" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Column Guide" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Workload" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Notes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module List" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Column Guide" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workload" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -719,7 +719,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Residential_Block_Low</t>
+          <t>/Game/Meshes/Placeholders/SM_Cube</t>
         </is>
       </c>
       <c r="G2" s="3" t="n">
@@ -893,7 +893,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Industrial_Warehouse</t>
+          <t>/Game/Meshes/Placeholders/SM_Cube</t>
         </is>
       </c>
       <c r="G5" s="3" t="n">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Service_Shopfront</t>
+          <t>/Game/Meshes/Placeholders/SM_Cube</t>
         </is>
       </c>
       <c r="G7" s="3" t="n">
@@ -1821,7 +1821,7 @@
       </c>
       <c r="F21" s="11" t="inlineStr">
         <is>
-          <t>/Game/Meshes/Modules/SM_Tree_Deciduous_Small</t>
+          <t>/Game/Meshes/Placeholders/SM_Cube</t>
         </is>
       </c>
       <c r="G21" s="12" t="n">
@@ -2916,7 +2916,7 @@
       </c>
     </row>
     <row r="2" ht="58" customHeight="1">
-      <c r="A2" s="27" t="inlineStr">
+      <c r="A2" s="43" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
@@ -2926,12 +2926,12 @@
           <t>The module's unique ID. PCG and the manifest refer to modules by this, never by DisplayName.</t>
         </is>
       </c>
-      <c r="C2" s="29" t="inlineStr">
+      <c r="C2" s="44" t="inlineStr">
         <is>
           <t>TA</t>
         </is>
       </c>
-      <c r="D2" s="29" t="inlineStr">
+      <c r="D2" s="44" t="inlineStr">
         <is>
           <t>REQUIRED</t>
         </is>
@@ -2941,7 +2941,7 @@
           <t>Must be unique. Format PREFIX_NNN. Never rename once PCG references it - renaming breaks every manifest that used it.</t>
         </is>
       </c>
-      <c r="F2" s="30" t="inlineStr">
+      <c r="F2" s="45" t="inlineStr">
         <is>
           <t>BLD_001</t>
         </is>
@@ -2980,7 +2980,7 @@
       </c>
     </row>
     <row r="4" ht="58" customHeight="1">
-      <c r="A4" s="27" t="inlineStr">
+      <c r="A4" s="43" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
@@ -2990,12 +2990,12 @@
           <t>Which of the six kit categories this belongs to. Used for grouping and category-level rules.</t>
         </is>
       </c>
-      <c r="C4" s="29" t="inlineStr">
+      <c r="C4" s="44" t="inlineStr">
         <is>
           <t>TA</t>
         </is>
       </c>
-      <c r="D4" s="29" t="inlineStr">
+      <c r="D4" s="44" t="inlineStr">
         <is>
           <t>REQUIRED</t>
         </is>
@@ -3005,14 +3005,14 @@
           <t>Must be one of the six existing categories. A typo creates a phantom category and the module silently drops out of its group.</t>
         </is>
       </c>
-      <c r="F4" s="30" t="inlineStr">
+      <c r="F4" s="45" t="inlineStr">
         <is>
           <t>Building</t>
         </is>
       </c>
     </row>
     <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="43" t="inlineStr">
         <is>
           <t>Zone</t>
         </is>
@@ -3022,12 +3022,12 @@
           <t>Which zone type a BUILDING belongs to. The manifest's zone ratios reference these.</t>
         </is>
       </c>
-      <c r="C5" s="29" t="inlineStr">
+      <c r="C5" s="44" t="inlineStr">
         <is>
           <t>TA</t>
         </is>
       </c>
-      <c r="D5" s="29" t="inlineStr">
+      <c r="D5" s="44" t="inlineStr">
         <is>
           <t>REQUIRED (buildings)</t>
         </is>
@@ -3037,14 +3037,14 @@
           <t>Residential / Industrial / Service for buildings. '-' for everything else. A building with '-' can never be placed.</t>
         </is>
       </c>
-      <c r="F5" s="30" t="inlineStr">
+      <c r="F5" s="45" t="inlineStr">
         <is>
           <t>Residential</t>
         </is>
       </c>
     </row>
     <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="27" t="inlineStr">
+      <c r="A6" s="43" t="inlineStr">
         <is>
           <t>Belt</t>
         </is>
@@ -3054,12 +3054,12 @@
           <t>Which belt this module is allowed on. A = hero belt, B = support, All = anywhere.</t>
         </is>
       </c>
-      <c r="C6" s="29" t="inlineStr">
+      <c r="C6" s="44" t="inlineStr">
         <is>
           <t>Artist</t>
         </is>
       </c>
-      <c r="D6" s="29" t="inlineStr">
+      <c r="D6" s="44" t="inlineStr">
         <is>
           <t>REQUIRED</t>
         </is>
@@ -3069,14 +3069,14 @@
           <t>A, B, or All. Belt C is cut from the project. Used to catch 'Belt A module used in Belt B'.</t>
         </is>
       </c>
-      <c r="F6" s="30" t="inlineStr">
+      <c r="F6" s="45" t="inlineStr">
         <is>
           <t>All</t>
         </is>
       </c>
     </row>
     <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="27" t="inlineStr">
+      <c r="A7" s="43" t="inlineStr">
         <is>
           <t>Mesh</t>
         </is>
@@ -3086,12 +3086,12 @@
           <t>Content Browser path to the asset PCG actually spawns. Without this, PCG has nothing to place.</t>
         </is>
       </c>
-      <c r="C7" s="29" t="inlineStr">
+      <c r="C7" s="44" t="inlineStr">
         <is>
           <t>Artist</t>
         </is>
       </c>
-      <c r="D7" s="29" t="inlineStr">
+      <c r="D7" s="44" t="inlineStr">
         <is>
           <t>REQUIRED</t>
         </is>
@@ -3101,14 +3101,14 @@
           <t>Must be a real path once the asset exists. Blank is allowed while unbuilt - the validator flags it as not-yet-ready, not an error.</t>
         </is>
       </c>
-      <c r="F7" s="30" t="inlineStr">
+      <c r="F7" s="45" t="inlineStr">
         <is>
           <t>/Game/Meshes/Modules/SM_Pipe_Elbow</t>
         </is>
       </c>
     </row>
     <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="27" t="inlineStr">
+      <c r="A8" s="43" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
@@ -3118,12 +3118,12 @@
           <t>How OFTEN this module gets picked compared to others in the same zone. 1.0 = common, 0.2 = rare.</t>
         </is>
       </c>
-      <c r="C8" s="29" t="inlineStr">
+      <c r="C8" s="44" t="inlineStr">
         <is>
           <t>Artist</t>
         </is>
       </c>
-      <c r="D8" s="29" t="inlineStr">
+      <c r="D8" s="44" t="inlineStr">
         <is>
           <t>REQUIRED</t>
         </is>
@@ -3133,7 +3133,7 @@
           <t>0.0 to 1.0. These are RELATIVE, not percentages - they do not need to sum to anything. Weight 0 means never placed. If every module is 1.0 the belt looks randomly shuffled rather than designed.</t>
         </is>
       </c>
-      <c r="F8" s="30" t="inlineStr">
+      <c r="F8" s="45" t="inlineStr">
         <is>
           <t>0.6</t>
         </is>

</xml_diff>